<commit_message>
Workbook fix: '=' -prefixed row labels forced to text (Excel read them as formulas -> #NAME?)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dossiers/athene/athene-quarterly-engine.xlsx
+++ b/dossiers/athene/athene-quarterly-engine.xlsx
@@ -665,9 +665,10 @@
       <c r="H10" s="7" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="8">
-        <f> Gross organic inflows</f>
-        <v/>
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>= Gross organic inflows</t>
+        </is>
       </c>
       <c r="B11" s="9">
         <f>SUM(B6:B10)</f>
@@ -721,9 +722,10 @@
       <c r="H12" s="7" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="8">
-        <f> TOTAL GROSS INFLOWS</f>
-        <v/>
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>= TOTAL GROSS INFLOWS</t>
+        </is>
       </c>
       <c r="B13" s="9">
         <f>B11+B12</f>
@@ -893,9 +895,10 @@
       <c r="H20" s="7" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="8">
-        <f> Total by owner</f>
-        <v/>
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>= Total by owner</t>
+        </is>
       </c>
       <c r="B21" s="9">
         <f>SUM(B18:B20)</f>
@@ -1013,9 +1016,10 @@
       <c r="H26" s="7" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="8">
-        <f> Total gross outflows</f>
-        <v/>
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>= Total gross outflows</t>
+        </is>
       </c>
       <c r="B27" s="9">
         <f>B25+B26</f>
@@ -1306,9 +1310,10 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="8">
-        <f> Net flows (inflows + outflows)</f>
-        <v/>
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>= Net flows (inflows + outflows)</t>
+        </is>
       </c>
       <c r="B40" s="9">
         <f>B13+B27</f>
@@ -1530,9 +1535,10 @@
       <c r="H49" s="7" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="8">
-        <f> Reserves — ending</f>
-        <v/>
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>= Reserves — ending</t>
+        </is>
       </c>
       <c r="B50" s="9">
         <f>SUM(B45:B49)</f>
@@ -1786,9 +1792,10 @@
       <c r="H60" s="7" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="8">
-        <f> ACRA reserves — ending</f>
-        <v/>
+      <c r="A61" s="8" t="inlineStr">
+        <is>
+          <t>= ACRA reserves — ending</t>
+        </is>
       </c>
       <c r="B61" s="9">
         <f>SUM(B56:B60)</f>
@@ -1920,9 +1927,10 @@
       <c r="H67" s="7" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="8">
-        <f> Total deferred annuities</f>
-        <v/>
+      <c r="A68" s="8" t="inlineStr">
+        <is>
+          <t>= Total deferred annuities</t>
+        </is>
       </c>
       <c r="B68" s="9">
         <f>B66+B67</f>
@@ -2030,9 +2038,10 @@
       <c r="H72" s="7" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="8">
-        <f> Total net reserve liabilities</f>
-        <v/>
+      <c r="A73" s="8" t="inlineStr">
+        <is>
+          <t>= Total net reserve liabilities</t>
+        </is>
       </c>
       <c r="B73" s="9">
         <f>B68+SUM(B69:B72)</f>
@@ -2170,9 +2179,10 @@
       <c r="H79" s="7" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="8">
-        <f> Net investment earnings</f>
-        <v/>
+      <c r="A80" s="8" t="inlineStr">
+        <is>
+          <t>= Net investment earnings</t>
+        </is>
       </c>
       <c r="B80" s="9">
         <f>B78+B79</f>
@@ -2252,9 +2262,10 @@
       <c r="H82" s="7" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="8">
-        <f> NET INVESTMENT SPREAD</f>
-        <v/>
+      <c r="A83" s="8" t="inlineStr">
+        <is>
+          <t>= NET INVESTMENT SPREAD</t>
+        </is>
       </c>
       <c r="B83" s="9">
         <f>SUM(B80:B82)</f>
@@ -2391,9 +2402,10 @@
       <c r="H87" s="7" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="8">
-        <f> SPREAD RELATED EARNINGS</f>
-        <v/>
+      <c r="A88" s="8" t="inlineStr">
+        <is>
+          <t>= SPREAD RELATED EARNINGS</t>
+        </is>
       </c>
       <c r="B88" s="9">
         <f>B83+B85+B86</f>
@@ -2700,9 +2712,10 @@
       <c r="H102" s="7" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="8">
-        <f> Average net invested assets</f>
-        <v/>
+      <c r="A103" s="8" t="inlineStr">
+        <is>
+          <t>= Average net invested assets</t>
+        </is>
       </c>
       <c r="B103" s="9">
         <f>B101+B102</f>

</xml_diff>

<commit_message>
Workbook fix: SRE formula off-by-one (referenced the check cell, ->#VALUE!); full ref audit clean
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dossiers/athene/athene-quarterly-engine.xlsx
+++ b/dossiers/athene/athene-quarterly-engine.xlsx
@@ -2408,27 +2408,27 @@
         </is>
       </c>
       <c r="B88" s="9">
-        <f>B83+B85+B86</f>
+        <f>B83+B86+B87</f>
         <v/>
       </c>
       <c r="C88" s="9">
-        <f>C83+C85+C86</f>
+        <f>C83+C86+C87</f>
         <v/>
       </c>
       <c r="D88" s="9">
-        <f>D83+D85+D86</f>
+        <f>D83+D86+D87</f>
         <v/>
       </c>
       <c r="E88" s="9">
-        <f>E83+E85+E86</f>
+        <f>E83+E86+E87</f>
         <v/>
       </c>
       <c r="F88" s="9">
-        <f>F83+F85+F86</f>
+        <f>F83+F86+F87</f>
         <v/>
       </c>
       <c r="G88" s="9">
-        <f>G83+G85+G86</f>
+        <f>G83+G86+G87</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Workbook fix: Checks master formula exceeded Excel's 8,192-char limit (316 COUNTIFs) — chunked into subtotals
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dossiers/athene/athene-quarterly-engine.xlsx
+++ b/dossiers/athene/athene-quarterly-engine.xlsx
@@ -8847,7 +8847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -8867,7 +8867,7 @@
         </is>
       </c>
       <c r="B3" s="8">
-        <f>COUNTIF('Engine'!B16,"FAIL")+COUNTIF('Engine'!C16,"FAIL")+COUNTIF('Engine'!D16,"FAIL")+COUNTIF('Engine'!E16,"FAIL")+COUNTIF('Engine'!F16,"FAIL")+COUNTIF('Engine'!G16,"FAIL")+COUNTIF('Engine'!B23,"FAIL")+COUNTIF('Engine'!C23,"FAIL")+COUNTIF('Engine'!D23,"FAIL")+COUNTIF('Engine'!E23,"FAIL")+COUNTIF('Engine'!F23,"FAIL")+COUNTIF('Engine'!G23,"FAIL")+COUNTIF('Engine'!B30,"FAIL")+COUNTIF('Engine'!C30,"FAIL")+COUNTIF('Engine'!D30,"FAIL")+COUNTIF('Engine'!E30,"FAIL")+COUNTIF('Engine'!F30,"FAIL")+COUNTIF('Engine'!G30,"FAIL")+COUNTIF('Engine'!B37,"FAIL")+COUNTIF('Engine'!C37,"FAIL")+COUNTIF('Engine'!D37,"FAIL")+COUNTIF('Engine'!E37,"FAIL")+COUNTIF('Engine'!F37,"FAIL")+COUNTIF('Engine'!G37,"FAIL")+COUNTIF('Engine'!B38,"FAIL")+COUNTIF('Engine'!C38,"FAIL")+COUNTIF('Engine'!D38,"FAIL")+COUNTIF('Engine'!E38,"FAIL")+COUNTIF('Engine'!F38,"FAIL")+COUNTIF('Engine'!G38,"FAIL")+COUNTIF('Engine'!B43,"FAIL")+COUNTIF('Engine'!C43,"FAIL")+COUNTIF('Engine'!D43,"FAIL")+COUNTIF('Engine'!E43,"FAIL")+COUNTIF('Engine'!F43,"FAIL")+COUNTIF('Engine'!G43,"FAIL")+COUNTIF('Engine'!B53,"FAIL")+COUNTIF('Engine'!C53,"FAIL")+COUNTIF('Engine'!D53,"FAIL")+COUNTIF('Engine'!E53,"FAIL")+COUNTIF('Engine'!F53,"FAIL")+COUNTIF('Engine'!G53,"FAIL")+COUNTIF('Engine'!C54,"FAIL")+COUNTIF('Engine'!D54,"FAIL")+COUNTIF('Engine'!E54,"FAIL")+COUNTIF('Engine'!F54,"FAIL")+COUNTIF('Engine'!G54,"FAIL")+COUNTIF('Engine'!B64,"FAIL")+COUNTIF('Engine'!C64,"FAIL")+COUNTIF('Engine'!D64,"FAIL")+COUNTIF('Engine'!E64,"FAIL")+COUNTIF('Engine'!F64,"FAIL")+COUNTIF('Engine'!G64,"FAIL")+COUNTIF('Engine'!B76,"FAIL")+COUNTIF('Engine'!C76,"FAIL")+COUNTIF('Engine'!D76,"FAIL")+COUNTIF('Engine'!E76,"FAIL")+COUNTIF('Engine'!F76,"FAIL")+COUNTIF('Engine'!G76,"FAIL")+COUNTIF('Engine'!B86,"FAIL")+COUNTIF('Engine'!C86,"FAIL")+COUNTIF('Engine'!D86,"FAIL")+COUNTIF('Engine'!E86,"FAIL")+COUNTIF('Engine'!F86,"FAIL")+COUNTIF('Engine'!G86,"FAIL")+COUNTIF('Engine'!B91,"FAIL")+COUNTIF('Engine'!C91,"FAIL")+COUNTIF('Engine'!D91,"FAIL")+COUNTIF('Engine'!E91,"FAIL")+COUNTIF('Engine'!F91,"FAIL")+COUNTIF('Engine'!G91,"FAIL")+COUNTIF('Engine'!B106,"FAIL")+COUNTIF('Engine'!C106,"FAIL")+COUNTIF('Engine'!D106,"FAIL")+COUNTIF('Engine'!E106,"FAIL")+COUNTIF('Engine'!F106,"FAIL")+COUNTIF('Engine'!G106,"FAIL")+COUNTIF('Engine'!B113,"FAIL")+COUNTIF('Engine'!C113,"FAIL")+COUNTIF('Engine'!D113,"FAIL")+COUNTIF('Engine'!E113,"FAIL")+COUNTIF('Engine'!F113,"FAIL")+COUNTIF('Engine'!G113,"FAIL")+COUNTIF('Engine'!B120,"FAIL")+COUNTIF('Engine'!C120,"FAIL")+COUNTIF('Engine'!D120,"FAIL")+COUNTIF('Engine'!E120,"FAIL")+COUNTIF('Engine'!F120,"FAIL")+COUNTIF('Engine'!G120,"FAIL")+COUNTIF('Engine'!B127,"FAIL")+COUNTIF('Engine'!C127,"FAIL")+COUNTIF('Engine'!D127,"FAIL")+COUNTIF('Engine'!E127,"FAIL")+COUNTIF('Engine'!F127,"FAIL")+COUNTIF('Engine'!G127,"FAIL")+COUNTIF('Engine'!B149,"FAIL")+COUNTIF('Engine'!C149,"FAIL")+COUNTIF('Engine'!D149,"FAIL")+COUNTIF('Engine'!E149,"FAIL")+COUNTIF('Engine'!F149,"FAIL")+COUNTIF('Engine'!G149,"FAIL")+COUNTIF('Engine'!B164,"FAIL")+COUNTIF('Engine'!C164,"FAIL")+COUNTIF('Engine'!D164,"FAIL")+COUNTIF('Engine'!E164,"FAIL")+COUNTIF('Engine'!F164,"FAIL")+COUNTIF('Engine'!G164,"FAIL")+COUNTIF('Engine'!B176,"FAIL")+COUNTIF('Engine'!C176,"FAIL")+COUNTIF('Engine'!D176,"FAIL")+COUNTIF('Engine'!E176,"FAIL")+COUNTIF('Engine'!F176,"FAIL")+COUNTIF('Engine'!G176,"FAIL")+COUNTIF('Engine'!B188,"FAIL")+COUNTIF('Engine'!C188,"FAIL")+COUNTIF('Engine'!D188,"FAIL")+COUNTIF('Engine'!E188,"FAIL")+COUNTIF('Engine'!F188,"FAIL")+COUNTIF('Engine'!G188,"FAIL")+COUNTIF('Engine'!B194,"FAIL")+COUNTIF('Engine'!C194,"FAIL")+COUNTIF('Engine'!D194,"FAIL")+COUNTIF('Engine'!E194,"FAIL")+COUNTIF('Engine'!F194,"FAIL")+COUNTIF('Engine'!G194,"FAIL")+COUNTIF('Engine'!B202,"FAIL")+COUNTIF('Engine'!C202,"FAIL")+COUNTIF('Engine'!D202,"FAIL")+COUNTIF('Engine'!E202,"FAIL")+COUNTIF('Engine'!F202,"FAIL")+COUNTIF('Engine'!G202,"FAIL")+COUNTIF('Engine'!B206,"FAIL")+COUNTIF('Engine'!C206,"FAIL")+COUNTIF('Engine'!D206,"FAIL")+COUNTIF('Engine'!E206,"FAIL")+COUNTIF('Engine'!F206,"FAIL")+COUNTIF('Engine'!G206,"FAIL")+COUNTIF('Engine-FY'!F7,"FAIL")+COUNTIF('Engine-FY'!F8,"FAIL")+COUNTIF('Engine-FY'!F9,"FAIL")+COUNTIF('Engine-FY'!F10,"FAIL")+COUNTIF('Engine-FY'!F11,"FAIL")+COUNTIF('Engine-FY'!F13,"FAIL")+COUNTIF('Engine-FY'!F15,"FAIL")+COUNTIF('Engine-FY'!B16,"FAIL")+COUNTIF('Engine-FY'!C16,"FAIL")+COUNTIF('Engine-FY'!D16,"FAIL")+COUNTIF('Engine-FY'!F19,"FAIL")+COUNTIF('Engine-FY'!F20,"FAIL")+COUNTIF('Engine-FY'!F21,"FAIL")+COUNTIF('Engine-FY'!B23,"FAIL")+COUNTIF('Engine-FY'!C23,"FAIL")+COUNTIF('Engine-FY'!D23,"FAIL")+COUNTIF('Engine-FY'!F26,"FAIL")+COUNTIF('Engine-FY'!F27,"FAIL")+COUNTIF('Engine-FY'!F29,"FAIL")+COUNTIF('Engine-FY'!B30,"FAIL")+COUNTIF('Engine-FY'!C30,"FAIL")+COUNTIF('Engine-FY'!D30,"FAIL")+COUNTIF('Engine-FY'!F32,"FAIL")+COUNTIF('Engine-FY'!F33,"FAIL")+COUNTIF('Engine-FY'!F34,"FAIL")+COUNTIF('Engine-FY'!F35,"FAIL")+COUNTIF('Engine-FY'!F36,"FAIL")+COUNTIF('Engine-FY'!B37,"FAIL")+COUNTIF('Engine-FY'!C37,"FAIL")+COUNTIF('Engine-FY'!D37,"FAIL")+COUNTIF('Engine-FY'!B38,"FAIL")+COUNTIF('Engine-FY'!C38,"FAIL")+COUNTIF('Engine-FY'!D38,"FAIL")+COUNTIF('Engine-FY'!F42,"FAIL")+COUNTIF('Engine-FY'!B43,"FAIL")+COUNTIF('Engine-FY'!C43,"FAIL")+COUNTIF('Engine-FY'!D43,"FAIL")+COUNTIF('Engine-FY'!F46,"FAIL")+COUNTIF('Engine-FY'!F47,"FAIL")+COUNTIF('Engine-FY'!F48,"FAIL")+COUNTIF('Engine-FY'!F49,"FAIL")+COUNTIF('Engine-FY'!F50,"FAIL")+COUNTIF('Engine-FY'!F52,"FAIL")+COUNTIF('Engine-FY'!B53,"FAIL")+COUNTIF('Engine-FY'!C53,"FAIL")+COUNTIF('Engine-FY'!D53,"FAIL")+COUNTIF('Engine-FY'!C54,"FAIL")+COUNTIF('Engine-FY'!D54,"FAIL")+COUNTIF('Engine-FY'!F57,"FAIL")+COUNTIF('Engine-FY'!F58,"FAIL")+COUNTIF('Engine-FY'!F59,"FAIL")+COUNTIF('Engine-FY'!F60,"FAIL")+COUNTIF('Engine-FY'!F61,"FAIL")+COUNTIF('Engine-FY'!F63,"FAIL")+COUNTIF('Engine-FY'!B64,"FAIL")+COUNTIF('Engine-FY'!C64,"FAIL")+COUNTIF('Engine-FY'!D64,"FAIL")+COUNTIF('Engine-FY'!F67,"FAIL")+COUNTIF('Engine-FY'!F68,"FAIL")+COUNTIF('Engine-FY'!F70,"FAIL")+COUNTIF('Engine-FY'!F71,"FAIL")+COUNTIF('Engine-FY'!F72,"FAIL")+COUNTIF('Engine-FY'!F73,"FAIL")+COUNTIF('Engine-FY'!F75,"FAIL")+COUNTIF('Engine-FY'!B76,"FAIL")+COUNTIF('Engine-FY'!C76,"FAIL")+COUNTIF('Engine-FY'!D76,"FAIL")+COUNTIF('Engine-FY'!F79,"FAIL")+COUNTIF('Engine-FY'!F80,"FAIL")+COUNTIF('Engine-FY'!F82,"FAIL")+COUNTIF('Engine-FY'!F83,"FAIL")+COUNTIF('Engine-FY'!F85,"FAIL")+COUNTIF('Engine-FY'!B86,"FAIL")+COUNTIF('Engine-FY'!C86,"FAIL")+COUNTIF('Engine-FY'!D86,"FAIL")+COUNTIF('Engine-FY'!F87,"FAIL")+COUNTIF('Engine-FY'!F88,"FAIL")+COUNTIF('Engine-FY'!F90,"FAIL")+COUNTIF('Engine-FY'!B91,"FAIL")+COUNTIF('Engine-FY'!C91,"FAIL")+COUNTIF('Engine-FY'!D91,"FAIL")+COUNTIF('Engine-FY'!F102,"FAIL")+COUNTIF('Engine-FY'!F103,"FAIL")+COUNTIF('Engine-FY'!B106,"FAIL")+COUNTIF('Engine-FY'!C106,"FAIL")+COUNTIF('Engine-FY'!D106,"FAIL")+COUNTIF('Engine-FY'!F109,"FAIL")+COUNTIF('Engine-FY'!F110,"FAIL")+COUNTIF('Engine-FY'!F111,"FAIL")+COUNTIF('Engine-FY'!F112,"FAIL")+COUNTIF('Engine-FY'!B113,"FAIL")+COUNTIF('Engine-FY'!C113,"FAIL")+COUNTIF('Engine-FY'!D113,"FAIL")+COUNTIF('Engine-FY'!F114,"FAIL")+COUNTIF('Engine-FY'!F115,"FAIL")+COUNTIF('Engine-FY'!F116,"FAIL")+COUNTIF('Engine-FY'!F117,"FAIL")+COUNTIF('Engine-FY'!F118,"FAIL")+COUNTIF('Engine-FY'!F119,"FAIL")+COUNTIF('Engine-FY'!B120,"FAIL")+COUNTIF('Engine-FY'!C120,"FAIL")+COUNTIF('Engine-FY'!D120,"FAIL")+COUNTIF('Engine-FY'!F122,"FAIL")+COUNTIF('Engine-FY'!F123,"FAIL")+COUNTIF('Engine-FY'!F124,"FAIL")+COUNTIF('Engine-FY'!B127,"FAIL")+COUNTIF('Engine-FY'!C127,"FAIL")+COUNTIF('Engine-FY'!D127,"FAIL")+COUNTIF('Engine-FY'!F130,"FAIL")+COUNTIF('Engine-FY'!F131,"FAIL")+COUNTIF('Engine-FY'!F133,"FAIL")+COUNTIF('Engine-FY'!F134,"FAIL")+COUNTIF('Engine-FY'!F135,"FAIL")+COUNTIF('Engine-FY'!F136,"FAIL")+COUNTIF('Engine-FY'!F138,"FAIL")+COUNTIF('Engine-FY'!F139,"FAIL")+COUNTIF('Engine-FY'!F140,"FAIL")+COUNTIF('Engine-FY'!F141,"FAIL")+COUNTIF('Engine-FY'!F142,"FAIL")+COUNTIF('Engine-FY'!F143,"FAIL")+COUNTIF('Engine-FY'!F145,"FAIL")+COUNTIF('Engine-FY'!F146,"FAIL")+COUNTIF('Engine-FY'!F148,"FAIL")+COUNTIF('Engine-FY'!B149,"FAIL")+COUNTIF('Engine-FY'!C149,"FAIL")+COUNTIF('Engine-FY'!D149,"FAIL")+COUNTIF('Engine-FY'!F152,"FAIL")+COUNTIF('Engine-FY'!F153,"FAIL")+COUNTIF('Engine-FY'!F154,"FAIL")+COUNTIF('Engine-FY'!F156,"FAIL")+COUNTIF('Engine-FY'!F157,"FAIL")+COUNTIF('Engine-FY'!F158,"FAIL")+COUNTIF('Engine-FY'!F159,"FAIL")+COUNTIF('Engine-FY'!F160,"FAIL")+COUNTIF('Engine-FY'!F163,"FAIL")+COUNTIF('Engine-FY'!B164,"FAIL")+COUNTIF('Engine-FY'!C164,"FAIL")+COUNTIF('Engine-FY'!D164,"FAIL")+COUNTIF('Engine-FY'!F167,"FAIL")+COUNTIF('Engine-FY'!F168,"FAIL")+COUNTIF('Engine-FY'!F169,"FAIL")+COUNTIF('Engine-FY'!F170,"FAIL")+COUNTIF('Engine-FY'!F171,"FAIL")+COUNTIF('Engine-FY'!F172,"FAIL")+COUNTIF('Engine-FY'!F173,"FAIL")+COUNTIF('Engine-FY'!F175,"FAIL")+COUNTIF('Engine-FY'!B176,"FAIL")+COUNTIF('Engine-FY'!C176,"FAIL")+COUNTIF('Engine-FY'!D176,"FAIL")+COUNTIF('Engine-FY'!F177,"FAIL")+COUNTIF('Engine-FY'!F178,"FAIL")+COUNTIF('Engine-FY'!F179,"FAIL")+COUNTIF('Engine-FY'!F180,"FAIL")+COUNTIF('Engine-FY'!F181,"FAIL")+COUNTIF('Engine-FY'!F183,"FAIL")+COUNTIF('Engine-FY'!F185,"FAIL")+COUNTIF('Engine-FY'!F187,"FAIL")+COUNTIF('Engine-FY'!B188,"FAIL")+COUNTIF('Engine-FY'!C188,"FAIL")+COUNTIF('Engine-FY'!D188,"FAIL")+COUNTIF('Engine-FY'!F189,"FAIL")+COUNTIF('Engine-FY'!F190,"FAIL")+COUNTIF('Engine-FY'!F191,"FAIL")+COUNTIF('Engine-FY'!F193,"FAIL")+COUNTIF('Engine-FY'!B194,"FAIL")+COUNTIF('Engine-FY'!C194,"FAIL")+COUNTIF('Engine-FY'!D194,"FAIL")+COUNTIF('Engine-FY'!F197,"FAIL")+COUNTIF('Engine-FY'!F198,"FAIL")+COUNTIF('Engine-FY'!F199,"FAIL")+COUNTIF('Engine-FY'!F201,"FAIL")+COUNTIF('Engine-FY'!B202,"FAIL")+COUNTIF('Engine-FY'!C202,"FAIL")+COUNTIF('Engine-FY'!D202,"FAIL")+COUNTIF('Engine-FY'!F203,"FAIL")+COUNTIF('Engine-FY'!F205,"FAIL")+COUNTIF('Engine-FY'!B206,"FAIL")+COUNTIF('Engine-FY'!C206,"FAIL")+COUNTIF('Engine-FY'!D206,"FAIL")</f>
+        <f>SUM(B8:B15)</f>
         <v/>
       </c>
     </row>
@@ -8876,6 +8876,94 @@
         <is>
           <t>Checks watched: 316 cells — totals cross-cuts, rollforward identities, continuity, SRE chain, derived spread, and the quarterly-vs-annual source audit.</t>
         </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>checks 1–40</t>
+        </is>
+      </c>
+      <c r="B8" s="2">
+        <f>COUNTIF('Engine'!B16,"FAIL")+COUNTIF('Engine'!C16,"FAIL")+COUNTIF('Engine'!D16,"FAIL")+COUNTIF('Engine'!E16,"FAIL")+COUNTIF('Engine'!F16,"FAIL")+COUNTIF('Engine'!G16,"FAIL")+COUNTIF('Engine'!B23,"FAIL")+COUNTIF('Engine'!C23,"FAIL")+COUNTIF('Engine'!D23,"FAIL")+COUNTIF('Engine'!E23,"FAIL")+COUNTIF('Engine'!F23,"FAIL")+COUNTIF('Engine'!G23,"FAIL")+COUNTIF('Engine'!B30,"FAIL")+COUNTIF('Engine'!C30,"FAIL")+COUNTIF('Engine'!D30,"FAIL")+COUNTIF('Engine'!E30,"FAIL")+COUNTIF('Engine'!F30,"FAIL")+COUNTIF('Engine'!G30,"FAIL")+COUNTIF('Engine'!B37,"FAIL")+COUNTIF('Engine'!C37,"FAIL")+COUNTIF('Engine'!D37,"FAIL")+COUNTIF('Engine'!E37,"FAIL")+COUNTIF('Engine'!F37,"FAIL")+COUNTIF('Engine'!G37,"FAIL")+COUNTIF('Engine'!B38,"FAIL")+COUNTIF('Engine'!C38,"FAIL")+COUNTIF('Engine'!D38,"FAIL")+COUNTIF('Engine'!E38,"FAIL")+COUNTIF('Engine'!F38,"FAIL")+COUNTIF('Engine'!G38,"FAIL")+COUNTIF('Engine'!B43,"FAIL")+COUNTIF('Engine'!C43,"FAIL")+COUNTIF('Engine'!D43,"FAIL")+COUNTIF('Engine'!E43,"FAIL")+COUNTIF('Engine'!F43,"FAIL")+COUNTIF('Engine'!G43,"FAIL")+COUNTIF('Engine'!B53,"FAIL")+COUNTIF('Engine'!C53,"FAIL")+COUNTIF('Engine'!D53,"FAIL")+COUNTIF('Engine'!E53,"FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>checks 41–80</t>
+        </is>
+      </c>
+      <c r="B9" s="2">
+        <f>COUNTIF('Engine'!F53,"FAIL")+COUNTIF('Engine'!G53,"FAIL")+COUNTIF('Engine'!C54,"FAIL")+COUNTIF('Engine'!D54,"FAIL")+COUNTIF('Engine'!E54,"FAIL")+COUNTIF('Engine'!F54,"FAIL")+COUNTIF('Engine'!G54,"FAIL")+COUNTIF('Engine'!B64,"FAIL")+COUNTIF('Engine'!C64,"FAIL")+COUNTIF('Engine'!D64,"FAIL")+COUNTIF('Engine'!E64,"FAIL")+COUNTIF('Engine'!F64,"FAIL")+COUNTIF('Engine'!G64,"FAIL")+COUNTIF('Engine'!B76,"FAIL")+COUNTIF('Engine'!C76,"FAIL")+COUNTIF('Engine'!D76,"FAIL")+COUNTIF('Engine'!E76,"FAIL")+COUNTIF('Engine'!F76,"FAIL")+COUNTIF('Engine'!G76,"FAIL")+COUNTIF('Engine'!B86,"FAIL")+COUNTIF('Engine'!C86,"FAIL")+COUNTIF('Engine'!D86,"FAIL")+COUNTIF('Engine'!E86,"FAIL")+COUNTIF('Engine'!F86,"FAIL")+COUNTIF('Engine'!G86,"FAIL")+COUNTIF('Engine'!B91,"FAIL")+COUNTIF('Engine'!C91,"FAIL")+COUNTIF('Engine'!D91,"FAIL")+COUNTIF('Engine'!E91,"FAIL")+COUNTIF('Engine'!F91,"FAIL")+COUNTIF('Engine'!G91,"FAIL")+COUNTIF('Engine'!B106,"FAIL")+COUNTIF('Engine'!C106,"FAIL")+COUNTIF('Engine'!D106,"FAIL")+COUNTIF('Engine'!E106,"FAIL")+COUNTIF('Engine'!F106,"FAIL")+COUNTIF('Engine'!G106,"FAIL")+COUNTIF('Engine'!B113,"FAIL")+COUNTIF('Engine'!C113,"FAIL")+COUNTIF('Engine'!D113,"FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>checks 81–120</t>
+        </is>
+      </c>
+      <c r="B10" s="2">
+        <f>COUNTIF('Engine'!E113,"FAIL")+COUNTIF('Engine'!F113,"FAIL")+COUNTIF('Engine'!G113,"FAIL")+COUNTIF('Engine'!B120,"FAIL")+COUNTIF('Engine'!C120,"FAIL")+COUNTIF('Engine'!D120,"FAIL")+COUNTIF('Engine'!E120,"FAIL")+COUNTIF('Engine'!F120,"FAIL")+COUNTIF('Engine'!G120,"FAIL")+COUNTIF('Engine'!B127,"FAIL")+COUNTIF('Engine'!C127,"FAIL")+COUNTIF('Engine'!D127,"FAIL")+COUNTIF('Engine'!E127,"FAIL")+COUNTIF('Engine'!F127,"FAIL")+COUNTIF('Engine'!G127,"FAIL")+COUNTIF('Engine'!B149,"FAIL")+COUNTIF('Engine'!C149,"FAIL")+COUNTIF('Engine'!D149,"FAIL")+COUNTIF('Engine'!E149,"FAIL")+COUNTIF('Engine'!F149,"FAIL")+COUNTIF('Engine'!G149,"FAIL")+COUNTIF('Engine'!B164,"FAIL")+COUNTIF('Engine'!C164,"FAIL")+COUNTIF('Engine'!D164,"FAIL")+COUNTIF('Engine'!E164,"FAIL")+COUNTIF('Engine'!F164,"FAIL")+COUNTIF('Engine'!G164,"FAIL")+COUNTIF('Engine'!B176,"FAIL")+COUNTIF('Engine'!C176,"FAIL")+COUNTIF('Engine'!D176,"FAIL")+COUNTIF('Engine'!E176,"FAIL")+COUNTIF('Engine'!F176,"FAIL")+COUNTIF('Engine'!G176,"FAIL")+COUNTIF('Engine'!B188,"FAIL")+COUNTIF('Engine'!C188,"FAIL")+COUNTIF('Engine'!D188,"FAIL")+COUNTIF('Engine'!E188,"FAIL")+COUNTIF('Engine'!F188,"FAIL")+COUNTIF('Engine'!G188,"FAIL")+COUNTIF('Engine'!B194,"FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>checks 121–160</t>
+        </is>
+      </c>
+      <c r="B11" s="2">
+        <f>COUNTIF('Engine'!C194,"FAIL")+COUNTIF('Engine'!D194,"FAIL")+COUNTIF('Engine'!E194,"FAIL")+COUNTIF('Engine'!F194,"FAIL")+COUNTIF('Engine'!G194,"FAIL")+COUNTIF('Engine'!B202,"FAIL")+COUNTIF('Engine'!C202,"FAIL")+COUNTIF('Engine'!D202,"FAIL")+COUNTIF('Engine'!E202,"FAIL")+COUNTIF('Engine'!F202,"FAIL")+COUNTIF('Engine'!G202,"FAIL")+COUNTIF('Engine'!B206,"FAIL")+COUNTIF('Engine'!C206,"FAIL")+COUNTIF('Engine'!D206,"FAIL")+COUNTIF('Engine'!E206,"FAIL")+COUNTIF('Engine'!F206,"FAIL")+COUNTIF('Engine'!G206,"FAIL")+COUNTIF('Engine-FY'!F7,"FAIL")+COUNTIF('Engine-FY'!F8,"FAIL")+COUNTIF('Engine-FY'!F9,"FAIL")+COUNTIF('Engine-FY'!F10,"FAIL")+COUNTIF('Engine-FY'!F11,"FAIL")+COUNTIF('Engine-FY'!F13,"FAIL")+COUNTIF('Engine-FY'!F15,"FAIL")+COUNTIF('Engine-FY'!B16,"FAIL")+COUNTIF('Engine-FY'!C16,"FAIL")+COUNTIF('Engine-FY'!D16,"FAIL")+COUNTIF('Engine-FY'!F19,"FAIL")+COUNTIF('Engine-FY'!F20,"FAIL")+COUNTIF('Engine-FY'!F21,"FAIL")+COUNTIF('Engine-FY'!B23,"FAIL")+COUNTIF('Engine-FY'!C23,"FAIL")+COUNTIF('Engine-FY'!D23,"FAIL")+COUNTIF('Engine-FY'!F26,"FAIL")+COUNTIF('Engine-FY'!F27,"FAIL")+COUNTIF('Engine-FY'!F29,"FAIL")+COUNTIF('Engine-FY'!B30,"FAIL")+COUNTIF('Engine-FY'!C30,"FAIL")+COUNTIF('Engine-FY'!D30,"FAIL")+COUNTIF('Engine-FY'!F32,"FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>checks 161–200</t>
+        </is>
+      </c>
+      <c r="B12" s="2">
+        <f>COUNTIF('Engine-FY'!F33,"FAIL")+COUNTIF('Engine-FY'!F34,"FAIL")+COUNTIF('Engine-FY'!F35,"FAIL")+COUNTIF('Engine-FY'!F36,"FAIL")+COUNTIF('Engine-FY'!B37,"FAIL")+COUNTIF('Engine-FY'!C37,"FAIL")+COUNTIF('Engine-FY'!D37,"FAIL")+COUNTIF('Engine-FY'!B38,"FAIL")+COUNTIF('Engine-FY'!C38,"FAIL")+COUNTIF('Engine-FY'!D38,"FAIL")+COUNTIF('Engine-FY'!F42,"FAIL")+COUNTIF('Engine-FY'!B43,"FAIL")+COUNTIF('Engine-FY'!C43,"FAIL")+COUNTIF('Engine-FY'!D43,"FAIL")+COUNTIF('Engine-FY'!F46,"FAIL")+COUNTIF('Engine-FY'!F47,"FAIL")+COUNTIF('Engine-FY'!F48,"FAIL")+COUNTIF('Engine-FY'!F49,"FAIL")+COUNTIF('Engine-FY'!F50,"FAIL")+COUNTIF('Engine-FY'!F52,"FAIL")+COUNTIF('Engine-FY'!B53,"FAIL")+COUNTIF('Engine-FY'!C53,"FAIL")+COUNTIF('Engine-FY'!D53,"FAIL")+COUNTIF('Engine-FY'!C54,"FAIL")+COUNTIF('Engine-FY'!D54,"FAIL")+COUNTIF('Engine-FY'!F57,"FAIL")+COUNTIF('Engine-FY'!F58,"FAIL")+COUNTIF('Engine-FY'!F59,"FAIL")+COUNTIF('Engine-FY'!F60,"FAIL")+COUNTIF('Engine-FY'!F61,"FAIL")+COUNTIF('Engine-FY'!F63,"FAIL")+COUNTIF('Engine-FY'!B64,"FAIL")+COUNTIF('Engine-FY'!C64,"FAIL")+COUNTIF('Engine-FY'!D64,"FAIL")+COUNTIF('Engine-FY'!F67,"FAIL")+COUNTIF('Engine-FY'!F68,"FAIL")+COUNTIF('Engine-FY'!F70,"FAIL")+COUNTIF('Engine-FY'!F71,"FAIL")+COUNTIF('Engine-FY'!F72,"FAIL")+COUNTIF('Engine-FY'!F73,"FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>checks 201–240</t>
+        </is>
+      </c>
+      <c r="B13" s="2">
+        <f>COUNTIF('Engine-FY'!F75,"FAIL")+COUNTIF('Engine-FY'!B76,"FAIL")+COUNTIF('Engine-FY'!C76,"FAIL")+COUNTIF('Engine-FY'!D76,"FAIL")+COUNTIF('Engine-FY'!F79,"FAIL")+COUNTIF('Engine-FY'!F80,"FAIL")+COUNTIF('Engine-FY'!F82,"FAIL")+COUNTIF('Engine-FY'!F83,"FAIL")+COUNTIF('Engine-FY'!F85,"FAIL")+COUNTIF('Engine-FY'!B86,"FAIL")+COUNTIF('Engine-FY'!C86,"FAIL")+COUNTIF('Engine-FY'!D86,"FAIL")+COUNTIF('Engine-FY'!F87,"FAIL")+COUNTIF('Engine-FY'!F88,"FAIL")+COUNTIF('Engine-FY'!F90,"FAIL")+COUNTIF('Engine-FY'!B91,"FAIL")+COUNTIF('Engine-FY'!C91,"FAIL")+COUNTIF('Engine-FY'!D91,"FAIL")+COUNTIF('Engine-FY'!F102,"FAIL")+COUNTIF('Engine-FY'!F103,"FAIL")+COUNTIF('Engine-FY'!B106,"FAIL")+COUNTIF('Engine-FY'!C106,"FAIL")+COUNTIF('Engine-FY'!D106,"FAIL")+COUNTIF('Engine-FY'!F109,"FAIL")+COUNTIF('Engine-FY'!F110,"FAIL")+COUNTIF('Engine-FY'!F111,"FAIL")+COUNTIF('Engine-FY'!F112,"FAIL")+COUNTIF('Engine-FY'!B113,"FAIL")+COUNTIF('Engine-FY'!C113,"FAIL")+COUNTIF('Engine-FY'!D113,"FAIL")+COUNTIF('Engine-FY'!F114,"FAIL")+COUNTIF('Engine-FY'!F115,"FAIL")+COUNTIF('Engine-FY'!F116,"FAIL")+COUNTIF('Engine-FY'!F117,"FAIL")+COUNTIF('Engine-FY'!F118,"FAIL")+COUNTIF('Engine-FY'!F119,"FAIL")+COUNTIF('Engine-FY'!B120,"FAIL")+COUNTIF('Engine-FY'!C120,"FAIL")+COUNTIF('Engine-FY'!D120,"FAIL")+COUNTIF('Engine-FY'!F122,"FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>checks 241–280</t>
+        </is>
+      </c>
+      <c r="B14" s="2">
+        <f>COUNTIF('Engine-FY'!F123,"FAIL")+COUNTIF('Engine-FY'!F124,"FAIL")+COUNTIF('Engine-FY'!B127,"FAIL")+COUNTIF('Engine-FY'!C127,"FAIL")+COUNTIF('Engine-FY'!D127,"FAIL")+COUNTIF('Engine-FY'!F130,"FAIL")+COUNTIF('Engine-FY'!F131,"FAIL")+COUNTIF('Engine-FY'!F133,"FAIL")+COUNTIF('Engine-FY'!F134,"FAIL")+COUNTIF('Engine-FY'!F135,"FAIL")+COUNTIF('Engine-FY'!F136,"FAIL")+COUNTIF('Engine-FY'!F138,"FAIL")+COUNTIF('Engine-FY'!F139,"FAIL")+COUNTIF('Engine-FY'!F140,"FAIL")+COUNTIF('Engine-FY'!F141,"FAIL")+COUNTIF('Engine-FY'!F142,"FAIL")+COUNTIF('Engine-FY'!F143,"FAIL")+COUNTIF('Engine-FY'!F145,"FAIL")+COUNTIF('Engine-FY'!F146,"FAIL")+COUNTIF('Engine-FY'!F148,"FAIL")+COUNTIF('Engine-FY'!B149,"FAIL")+COUNTIF('Engine-FY'!C149,"FAIL")+COUNTIF('Engine-FY'!D149,"FAIL")+COUNTIF('Engine-FY'!F152,"FAIL")+COUNTIF('Engine-FY'!F153,"FAIL")+COUNTIF('Engine-FY'!F154,"FAIL")+COUNTIF('Engine-FY'!F156,"FAIL")+COUNTIF('Engine-FY'!F157,"FAIL")+COUNTIF('Engine-FY'!F158,"FAIL")+COUNTIF('Engine-FY'!F159,"FAIL")+COUNTIF('Engine-FY'!F160,"FAIL")+COUNTIF('Engine-FY'!F163,"FAIL")+COUNTIF('Engine-FY'!B164,"FAIL")+COUNTIF('Engine-FY'!C164,"FAIL")+COUNTIF('Engine-FY'!D164,"FAIL")+COUNTIF('Engine-FY'!F167,"FAIL")+COUNTIF('Engine-FY'!F168,"FAIL")+COUNTIF('Engine-FY'!F169,"FAIL")+COUNTIF('Engine-FY'!F170,"FAIL")+COUNTIF('Engine-FY'!F171,"FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>checks 281–316</t>
+        </is>
+      </c>
+      <c r="B15" s="2">
+        <f>COUNTIF('Engine-FY'!F172,"FAIL")+COUNTIF('Engine-FY'!F173,"FAIL")+COUNTIF('Engine-FY'!F175,"FAIL")+COUNTIF('Engine-FY'!B176,"FAIL")+COUNTIF('Engine-FY'!C176,"FAIL")+COUNTIF('Engine-FY'!D176,"FAIL")+COUNTIF('Engine-FY'!F177,"FAIL")+COUNTIF('Engine-FY'!F178,"FAIL")+COUNTIF('Engine-FY'!F179,"FAIL")+COUNTIF('Engine-FY'!F180,"FAIL")+COUNTIF('Engine-FY'!F181,"FAIL")+COUNTIF('Engine-FY'!F183,"FAIL")+COUNTIF('Engine-FY'!F185,"FAIL")+COUNTIF('Engine-FY'!F187,"FAIL")+COUNTIF('Engine-FY'!B188,"FAIL")+COUNTIF('Engine-FY'!C188,"FAIL")+COUNTIF('Engine-FY'!D188,"FAIL")+COUNTIF('Engine-FY'!F189,"FAIL")+COUNTIF('Engine-FY'!F190,"FAIL")+COUNTIF('Engine-FY'!F191,"FAIL")+COUNTIF('Engine-FY'!F193,"FAIL")+COUNTIF('Engine-FY'!B194,"FAIL")+COUNTIF('Engine-FY'!C194,"FAIL")+COUNTIF('Engine-FY'!D194,"FAIL")+COUNTIF('Engine-FY'!F197,"FAIL")+COUNTIF('Engine-FY'!F198,"FAIL")+COUNTIF('Engine-FY'!F199,"FAIL")+COUNTIF('Engine-FY'!F201,"FAIL")+COUNTIF('Engine-FY'!B202,"FAIL")+COUNTIF('Engine-FY'!C202,"FAIL")+COUNTIF('Engine-FY'!D202,"FAIL")+COUNTIF('Engine-FY'!F203,"FAIL")+COUNTIF('Engine-FY'!F205,"FAIL")+COUNTIF('Engine-FY'!B206,"FAIL")+COUNTIF('Engine-FY'!C206,"FAIL")+COUNTIF('Engine-FY'!D206,"FAIL")</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>